<commit_message>
Added manual course ENST-443 and bug fixes
</commit_message>
<xml_diff>
--- a/data_raw/Template_for_Adding_Courses_to_Sustainability_Course_Finder.xlsx
+++ b/data_raw/Template_for_Adding_Courses_to_Sustainability_Course_Finder.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\SustainabilityCourseFinder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fy916/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CD92707-8B2C-4F2F-BBC7-0EAB03730052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C4E899-652D-FE4E-AF7C-8A82E553F558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="8170" xr2:uid="{3E9B7C92-6739-1340-9EDD-02531B8302F5}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="41120" windowHeight="25420" xr2:uid="{3E9B7C92-6739-1340-9EDD-02531B8302F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="48">
   <si>
     <t>Andrew and Erna Viterbi School of Engineering</t>
   </si>
@@ -147,6 +147,39 @@
   </si>
   <si>
     <t>Update Description</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>completed</t>
+  </si>
+  <si>
+    <t>An immersive course in qualitative field research, justice-based policy analysis and effective climate communication through study of the UN Framework Convention on Climate Change negotiations.</t>
+  </si>
+  <si>
+    <t>ENST</t>
+  </si>
+  <si>
+    <t>ENST-443</t>
+  </si>
+  <si>
+    <t>Global Climate Negotiations: Research and Communication</t>
+  </si>
+  <si>
+    <t>Gibson, Shannon</t>
+  </si>
+  <si>
+    <t>33071D</t>
+  </si>
+  <si>
+    <t>F25</t>
+  </si>
+  <si>
+    <t>AY26</t>
+  </si>
+  <si>
+    <t>Dana and David Dornsife College of Letters, Arts and Sciences</t>
   </si>
 </sst>
 </file>
@@ -269,9 +302,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -309,7 +342,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -415,7 +448,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -557,7 +590,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -565,11 +598,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8B90C02-862D-8944-8647-8139FC139BF2}">
-  <dimension ref="A1:N4"/>
-  <sheetFormatPr defaultColWidth="11.1640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:O5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.83203125" style="5" customWidth="1"/>
-    <col min="2" max="2" width="11.1640625" style="5"/>
+    <col min="2" max="2" width="37.83203125" style="5" customWidth="1"/>
     <col min="3" max="3" width="16" style="5" customWidth="1"/>
     <col min="4" max="9" width="11.1640625" style="5"/>
     <col min="10" max="10" width="75.1640625" style="5" customWidth="1"/>
@@ -579,7 +612,7 @@
     <col min="14" max="16384" width="11.1640625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" s="1" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -622,8 +655,11 @@
       <c r="N1" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="O1" s="1" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>36</v>
       </c>
@@ -663,8 +699,11 @@
       <c r="M2" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="O2" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>36</v>
       </c>
@@ -707,8 +746,11 @@
       <c r="N3" s="5">
         <v>48</v>
       </c>
+      <c r="O3" s="5" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="4" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>16</v>
       </c>
@@ -750,10 +792,55 @@
       </c>
       <c r="N4" s="7">
         <v>966</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="5">
+        <v>1</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="N5" s="5">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>